<commit_message>
Update IG-workflows action to use feature branch 2468f0f6190c5ec856812da8b0745bd4ebcc9f8d
</commit_message>
<xml_diff>
--- a/nriss-patch-1/ig/StructureDefinition-mesures-bundle-flux-alimentation-biologie.xlsx
+++ b/nriss-patch-1/ig/StructureDefinition-mesures-bundle-flux-alimentation-biologie.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-23T17:05:55+00:00</t>
+    <t>2026-10-07T08:01:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>France</t>
+    <t>France (la)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>